<commit_message>
reduce air res bleed
</commit_message>
<xml_diff>
--- a/stat_graphs/Vehicle Stats.xlsx
+++ b/stat_graphs/Vehicle Stats.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Planes" sheetId="1" state="visible" r:id="rId3"/>
@@ -10845,7 +10845,7 @@
         <v>2</v>
       </c>
       <c r="E70" s="0" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
modified felix physics stats
</commit_message>
<xml_diff>
--- a/stat_graphs/Vehicle Stats.xlsx
+++ b/stat_graphs/Vehicle Stats.xlsx
@@ -645,7 +645,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -747,6 +747,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -9787,7 +9791,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F80"/>
+  <dimension ref="A1:F79"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="19.33"/>
@@ -9866,7 +9870,7 @@
       <c r="E7" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="F7" s="1"/>
+      <c r="F7" s="26"/>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="n">
@@ -10097,7 +10101,7 @@
       <c r="E22" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="F22" s="1"/>
+      <c r="F22" s="26"/>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="n">
@@ -10233,7 +10237,7 @@
       <c r="E32" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="F32" s="1"/>
+      <c r="F32" s="26"/>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="n">
@@ -10578,7 +10582,7 @@
       <c r="E53" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="F53" s="1"/>
+      <c r="F53" s="26"/>
     </row>
     <row r="54" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="n">
@@ -10831,210 +10835,191 @@
     </row>
     <row r="70" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="0" t="n">
-        <v>240</v>
+        <v>360.5</v>
       </c>
       <c r="B70" s="0" t="n">
         <f aca="false">A70*$A$2*$D$2</f>
-        <v>8.333333334</v>
+        <v>12.5173611121125</v>
       </c>
       <c r="C70" s="0" t="n">
         <f aca="false">B70*$C$2</f>
-        <v>0.4166666667</v>
+        <v>0.625868055605625</v>
       </c>
       <c r="D70" s="0" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E70" s="0" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="0" t="n">
-        <v>360.5</v>
+        <v>481</v>
       </c>
       <c r="B71" s="0" t="n">
         <f aca="false">A71*$A$2*$D$2</f>
-        <v>12.5173611121125</v>
+        <v>16.701388890225</v>
       </c>
       <c r="C71" s="0" t="n">
         <f aca="false">B71*$C$2</f>
-        <v>0.625868055605625</v>
+        <v>0.83506944451125</v>
       </c>
       <c r="D71" s="0" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E71" s="0" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="0" t="n">
-        <v>481</v>
+        <v>601.5</v>
       </c>
       <c r="B72" s="0" t="n">
         <f aca="false">A72*$A$2*$D$2</f>
-        <v>16.701388890225</v>
+        <v>20.8854166683375</v>
       </c>
       <c r="C72" s="0" t="n">
         <f aca="false">B72*$C$2</f>
-        <v>0.83506944451125</v>
+        <v>1.04427083341688</v>
       </c>
       <c r="D72" s="0" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E72" s="0" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="0" t="n">
-        <v>601.5</v>
+        <v>722</v>
       </c>
       <c r="B73" s="0" t="n">
         <f aca="false">A73*$A$2*$D$2</f>
-        <v>20.8854166683375</v>
+        <v>25.06944444645</v>
       </c>
       <c r="C73" s="0" t="n">
         <f aca="false">B73*$C$2</f>
-        <v>1.04427083341688</v>
+        <v>1.2534722223225</v>
       </c>
       <c r="D73" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="E73" s="0" t="n">
         <v>11</v>
-      </c>
-      <c r="E73" s="0" t="n">
-        <v>13</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="0" t="n">
-        <v>722</v>
+        <v>842.5</v>
       </c>
       <c r="B74" s="0" t="n">
         <f aca="false">A74*$A$2*$D$2</f>
-        <v>25.06944444645</v>
+        <v>29.2534722245625</v>
       </c>
       <c r="C74" s="0" t="n">
         <f aca="false">B74*$C$2</f>
-        <v>1.2534722223225</v>
+        <v>1.46267361122813</v>
       </c>
       <c r="D74" s="0" t="n">
-        <v>11.8</v>
+        <v>14</v>
       </c>
       <c r="E74" s="0" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="0" t="n">
-        <v>842.5</v>
+        <v>963</v>
       </c>
       <c r="B75" s="0" t="n">
         <f aca="false">A75*$A$2*$D$2</f>
-        <v>29.2534722245625</v>
+        <v>33.437500002675</v>
       </c>
       <c r="C75" s="0" t="n">
         <f aca="false">B75*$C$2</f>
-        <v>1.46267361122813</v>
+        <v>1.67187500013375</v>
       </c>
       <c r="D75" s="0" t="n">
-        <v>12.3</v>
+        <v>15</v>
       </c>
       <c r="E75" s="0" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="0" t="n">
-        <v>963</v>
+        <v>1083.5</v>
       </c>
       <c r="B76" s="0" t="n">
         <f aca="false">A76*$A$2*$D$2</f>
-        <v>33.437500002675</v>
+        <v>37.6215277807875</v>
       </c>
       <c r="C76" s="0" t="n">
         <f aca="false">B76*$C$2</f>
-        <v>1.67187500013375</v>
+        <v>1.88107638903938</v>
       </c>
       <c r="D76" s="0" t="n">
-        <v>12.9</v>
+        <v>14</v>
       </c>
       <c r="E76" s="0" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="0" t="n">
-        <v>1083.5</v>
+        <v>1204</v>
       </c>
       <c r="B77" s="0" t="n">
         <f aca="false">A77*$A$2*$D$2</f>
-        <v>37.6215277807875</v>
+        <v>41.8055555589</v>
       </c>
       <c r="C77" s="0" t="n">
         <f aca="false">B77*$C$2</f>
-        <v>1.88107638903938</v>
+        <v>2.090277777945</v>
       </c>
       <c r="D77" s="0" t="n">
-        <v>12.1</v>
+        <v>12</v>
       </c>
       <c r="E77" s="0" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="0" t="n">
-        <v>1204</v>
+        <v>1324.5</v>
       </c>
       <c r="B78" s="0" t="n">
         <f aca="false">A78*$A$2*$D$2</f>
-        <v>41.8055555589</v>
+        <v>45.9895833370125</v>
       </c>
       <c r="C78" s="0" t="n">
         <f aca="false">B78*$C$2</f>
-        <v>2.090277777945</v>
+        <v>2.29947916685063</v>
       </c>
       <c r="D78" s="0" t="n">
         <v>9</v>
       </c>
       <c r="E78" s="0" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="0" t="n">
-        <v>1324.5</v>
+        <v>1445</v>
       </c>
       <c r="B79" s="0" t="n">
         <f aca="false">A79*$A$2*$D$2</f>
-        <v>45.9895833370125</v>
+        <v>50.173611115125</v>
       </c>
       <c r="C79" s="0" t="n">
         <f aca="false">B79*$C$2</f>
-        <v>2.29947916685063</v>
+        <v>2.50868055575625</v>
       </c>
       <c r="D79" s="0" t="n">
-        <v>7.3</v>
+        <v>6</v>
       </c>
       <c r="E79" s="0" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A80" s="0" t="n">
-        <v>1445</v>
-      </c>
-      <c r="B80" s="0" t="n">
-        <f aca="false">A80*$A$2*$D$2</f>
-        <v>50.173611115125</v>
-      </c>
-      <c r="C80" s="0" t="n">
-        <f aca="false">B80*$C$2</f>
-        <v>2.50868055575625</v>
-      </c>
-      <c r="D80" s="0" t="n">
-        <v>5.6</v>
-      </c>
-      <c r="E80" s="0" t="n">
         <v>2</v>
       </c>
     </row>
@@ -11111,10 +11096,10 @@
       <c r="C4" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="27" t="s">
         <v>98</v>
       </c>
-      <c r="E4" s="27" t="s">
+      <c r="E4" s="28" t="s">
         <v>104</v>
       </c>
       <c r="F4" s="1" t="s">
@@ -11126,13 +11111,13 @@
       <c r="H4" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="I4" s="26" t="s">
+      <c r="I4" s="27" t="s">
         <v>108</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="K4" s="26" t="s">
+      <c r="K4" s="27" t="s">
         <v>110</v>
       </c>
     </row>
@@ -11345,7 +11330,7 @@
       <c r="A10" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="B10" s="28" t="n">
+      <c r="B10" s="29" t="n">
         <v>6170</v>
       </c>
       <c r="C10" s="9" t="n">

</xml_diff>